<commit_message>
Frame name changed to dev
</commit_message>
<xml_diff>
--- a/OctopusSaas_26_06_2026/Test data/read.xlsx
+++ b/OctopusSaas_26_06_2026/Test data/read.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/35140d9111016f1f/Desktop/Octopus saas/Excwl sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32CD2F2E-382B-4F7D-B383-FFC0A9368A59}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:801_{0A411D91-5D81-46AE-BAA6-DBE729FACD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4C2F324-12B7-45F4-8566-7C1CE3AA4C28}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="463">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1429,6 +1429,12 @@
   </si>
   <si>
     <t>12</t>
+  </si>
+  <si>
+    <t>Email name</t>
+  </si>
+  <si>
+    <t>ballu</t>
   </si>
 </sst>
 </file>
@@ -1516,6 +1522,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3912,7 +3922,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="6" bestFit="1" customWidth="1"/>
@@ -4150,6 +4160,19 @@
       </c>
       <c r="G22" s="8" t="s">
         <v>460</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B25" s="6" t="s">
+        <v>462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>